<commit_message>
3.2 (new placeholdedrs protocol)
</commit_message>
<xml_diff>
--- a/main/cars/templates/НОВЫЕ/ТЗ по неприменимости 1.xlsx
+++ b/main/cars/templates/НОВЫЕ/ТЗ по неприменимости 1.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="219">
   <si>
     <t>не применяется (ТС не используется для коммерческих перевозок)</t>
   </si>
@@ -1197,7 +1197,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="115">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1367,158 +1367,172 @@
     </xf>
     <xf numFmtId="49" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -1799,13 +1813,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M292"/>
+  <dimension ref="A1:M293"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" customWidth="1"/>
     <col min="2" max="2" width="7.28515625" customWidth="1"/>
     <col min="3" max="3" width="14.85546875" customWidth="1"/>
     <col min="4" max="4" width="102.28515625" customWidth="1"/>
+    <col min="6" max="6" width="28.140625" customWidth="1"/>
+    <col min="7" max="7" width="90.5703125" customWidth="1"/>
+    <col min="8" max="8" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -1824,10 +1841,10 @@
       <c r="M1" s="1"/>
     </row>
     <row r="2" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="97">
+      <c r="A2" s="76">
         <v>0</v>
       </c>
-      <c r="B2" s="100" t="s">
+      <c r="B2" s="79" t="s">
         <v>211</v>
       </c>
       <c r="C2" s="6" t="s">
@@ -1847,8 +1864,8 @@
       <c r="M2" s="1"/>
     </row>
     <row r="3" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="98"/>
-      <c r="B3" s="101"/>
+      <c r="A3" s="77"/>
+      <c r="B3" s="80"/>
       <c r="C3" s="7" t="s">
         <v>10</v>
       </c>
@@ -1866,8 +1883,8 @@
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="99"/>
-      <c r="B4" s="102"/>
+      <c r="A4" s="78"/>
+      <c r="B4" s="81"/>
       <c r="C4" s="8" t="s">
         <v>11</v>
       </c>
@@ -1885,10 +1902,10 @@
       <c r="M4" s="1"/>
     </row>
     <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="97">
+      <c r="A5" s="76">
         <v>1</v>
       </c>
-      <c r="B5" s="104" t="s">
+      <c r="B5" s="82" t="s">
         <v>1</v>
       </c>
       <c r="C5" s="50" t="s">
@@ -1908,8 +1925,8 @@
       <c r="M5" s="1"/>
     </row>
     <row r="6" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="98"/>
-      <c r="B6" s="105"/>
+      <c r="A6" s="77"/>
+      <c r="B6" s="83"/>
       <c r="C6" s="51" t="s">
         <v>16</v>
       </c>
@@ -1927,8 +1944,8 @@
       <c r="M6" s="1"/>
     </row>
     <row r="7" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="108"/>
-      <c r="B7" s="106"/>
+      <c r="A7" s="86"/>
+      <c r="B7" s="84"/>
       <c r="C7" s="51" t="s">
         <v>17</v>
       </c>
@@ -1946,8 +1963,8 @@
       <c r="M7" s="1"/>
     </row>
     <row r="8" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="99"/>
-      <c r="B8" s="107"/>
+      <c r="A8" s="78"/>
+      <c r="B8" s="85"/>
       <c r="C8" s="49" t="s">
         <v>212</v>
       </c>
@@ -1988,13 +2005,13 @@
       <c r="M9" s="1"/>
     </row>
     <row r="10" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="89" t="s">
+      <c r="A10" s="67" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="61" t="s">
+      <c r="B10" s="70" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="61" t="s">
+      <c r="C10" s="70" t="s">
         <v>19</v>
       </c>
       <c r="D10" s="13" t="s">
@@ -2011,9 +2028,9 @@
       <c r="M10" s="1"/>
     </row>
     <row r="11" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="90"/>
-      <c r="B11" s="67"/>
-      <c r="C11" s="67"/>
+      <c r="A11" s="68"/>
+      <c r="B11" s="71"/>
+      <c r="C11" s="71"/>
       <c r="D11" s="14" t="s">
         <v>7</v>
       </c>
@@ -2028,9 +2045,9 @@
       <c r="M11" s="1"/>
     </row>
     <row r="12" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="90"/>
-      <c r="B12" s="67"/>
-      <c r="C12" s="67" t="s">
+      <c r="A12" s="68"/>
+      <c r="B12" s="71"/>
+      <c r="C12" s="71" t="s">
         <v>20</v>
       </c>
       <c r="D12" s="10" t="s">
@@ -2047,9 +2064,9 @@
       <c r="M12" s="1"/>
     </row>
     <row r="13" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="103"/>
-      <c r="B13" s="62"/>
-      <c r="C13" s="62"/>
+      <c r="A13" s="69"/>
+      <c r="B13" s="72"/>
+      <c r="C13" s="72"/>
       <c r="D13" s="15" t="s">
         <v>8</v>
       </c>
@@ -2064,10 +2081,10 @@
       <c r="M13" s="1"/>
     </row>
     <row r="14" spans="1:13" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="A14" s="89" t="s">
+      <c r="A14" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="61" t="s">
+      <c r="B14" s="70" t="s">
         <v>14</v>
       </c>
       <c r="C14" s="6" t="s">
@@ -2087,8 +2104,8 @@
       <c r="M14" s="1"/>
     </row>
     <row r="15" spans="1:13" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="A15" s="90"/>
-      <c r="B15" s="67"/>
+      <c r="A15" s="68"/>
+      <c r="B15" s="71"/>
       <c r="C15" s="7" t="s">
         <v>22</v>
       </c>
@@ -2106,8 +2123,8 @@
       <c r="M15" s="1"/>
     </row>
     <row r="16" spans="1:13" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="A16" s="90"/>
-      <c r="B16" s="67"/>
+      <c r="A16" s="68"/>
+      <c r="B16" s="71"/>
       <c r="C16" s="7" t="s">
         <v>23</v>
       </c>
@@ -2125,8 +2142,8 @@
       <c r="M16" s="1"/>
     </row>
     <row r="17" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="90"/>
-      <c r="B17" s="67"/>
+      <c r="A17" s="68"/>
+      <c r="B17" s="71"/>
       <c r="C17" s="7" t="s">
         <v>24</v>
       </c>
@@ -2144,8 +2161,8 @@
       <c r="M17" s="1"/>
     </row>
     <row r="18" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="90"/>
-      <c r="B18" s="67"/>
+      <c r="A18" s="68"/>
+      <c r="B18" s="71"/>
       <c r="C18" s="7" t="s">
         <v>25</v>
       </c>
@@ -2163,8 +2180,8 @@
       <c r="M18" s="1"/>
     </row>
     <row r="19" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="90"/>
-      <c r="B19" s="67"/>
+      <c r="A19" s="68"/>
+      <c r="B19" s="71"/>
       <c r="C19" s="7" t="s">
         <v>26</v>
       </c>
@@ -2182,8 +2199,8 @@
       <c r="M19" s="1"/>
     </row>
     <row r="20" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="90"/>
-      <c r="B20" s="67"/>
+      <c r="A20" s="68"/>
+      <c r="B20" s="71"/>
       <c r="C20" s="7" t="s">
         <v>27</v>
       </c>
@@ -2201,8 +2218,8 @@
       <c r="M20" s="1"/>
     </row>
     <row r="21" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="103"/>
-      <c r="B21" s="62"/>
+      <c r="A21" s="69"/>
+      <c r="B21" s="72"/>
       <c r="C21" s="17" t="s">
         <v>12</v>
       </c>
@@ -2220,10 +2237,10 @@
       <c r="M21" s="1"/>
     </row>
     <row r="22" spans="1:13" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="A22" s="89" t="s">
+      <c r="A22" s="67" t="s">
         <v>30</v>
       </c>
-      <c r="B22" s="61" t="s">
+      <c r="B22" s="70" t="s">
         <v>31</v>
       </c>
       <c r="C22" s="6" t="s">
@@ -2243,9 +2260,9 @@
       <c r="M22" s="1"/>
     </row>
     <row r="23" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="90"/>
-      <c r="B23" s="67"/>
-      <c r="C23" s="67" t="s">
+      <c r="A23" s="68"/>
+      <c r="B23" s="71"/>
+      <c r="C23" s="71" t="s">
         <v>29</v>
       </c>
       <c r="D23" s="26" t="s">
@@ -2262,9 +2279,9 @@
       <c r="M23" s="1"/>
     </row>
     <row r="24" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="103"/>
-      <c r="B24" s="62"/>
-      <c r="C24" s="62"/>
+      <c r="A24" s="69"/>
+      <c r="B24" s="72"/>
+      <c r="C24" s="72"/>
       <c r="D24" s="30" t="s">
         <v>8</v>
       </c>
@@ -2279,10 +2296,10 @@
       <c r="M24" s="1"/>
     </row>
     <row r="25" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="89" t="s">
+      <c r="A25" s="67" t="s">
         <v>35</v>
       </c>
-      <c r="B25" s="61" t="s">
+      <c r="B25" s="70" t="s">
         <v>36</v>
       </c>
       <c r="C25" s="6" t="s">
@@ -2302,8 +2319,8 @@
       <c r="M25" s="1"/>
     </row>
     <row r="26" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="90"/>
-      <c r="B26" s="67"/>
+      <c r="A26" s="68"/>
+      <c r="B26" s="71"/>
       <c r="C26" s="7" t="s">
         <v>33</v>
       </c>
@@ -2321,8 +2338,8 @@
       <c r="M26" s="1"/>
     </row>
     <row r="27" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="103"/>
-      <c r="B27" s="62"/>
+      <c r="A27" s="69"/>
+      <c r="B27" s="72"/>
       <c r="C27" s="17" t="s">
         <v>34</v>
       </c>
@@ -2340,10 +2357,10 @@
       <c r="M27" s="1"/>
     </row>
     <row r="28" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="92" t="s">
+      <c r="A28" s="87" t="s">
         <v>37</v>
       </c>
-      <c r="B28" s="95" t="s">
+      <c r="B28" s="90" t="s">
         <v>38</v>
       </c>
       <c r="C28" s="18" t="s">
@@ -2363,9 +2380,9 @@
       <c r="M28" s="1"/>
     </row>
     <row r="29" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="93"/>
-      <c r="B29" s="96"/>
-      <c r="C29" s="67" t="s">
+      <c r="A29" s="88"/>
+      <c r="B29" s="91"/>
+      <c r="C29" s="71" t="s">
         <v>40</v>
       </c>
       <c r="D29" s="40" t="s">
@@ -2382,9 +2399,9 @@
       <c r="M29" s="1"/>
     </row>
     <row r="30" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="93"/>
-      <c r="B30" s="96"/>
-      <c r="C30" s="67"/>
+      <c r="A30" s="88"/>
+      <c r="B30" s="91"/>
+      <c r="C30" s="71"/>
       <c r="D30" s="16" t="s">
         <v>8</v>
       </c>
@@ -2399,9 +2416,9 @@
       <c r="M30" s="1"/>
     </row>
     <row r="31" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A31" s="93"/>
-      <c r="B31" s="96"/>
-      <c r="C31" s="67" t="s">
+      <c r="A31" s="88"/>
+      <c r="B31" s="91"/>
+      <c r="C31" s="71" t="s">
         <v>41</v>
       </c>
       <c r="D31" s="40" t="s">
@@ -2418,9 +2435,9 @@
       <c r="M31" s="1"/>
     </row>
     <row r="32" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A32" s="93"/>
-      <c r="B32" s="96"/>
-      <c r="C32" s="67"/>
+      <c r="A32" s="88"/>
+      <c r="B32" s="91"/>
+      <c r="C32" s="71"/>
       <c r="D32" s="28" t="s">
         <v>149</v>
       </c>
@@ -2435,9 +2452,9 @@
       <c r="M32" s="1"/>
     </row>
     <row r="33" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A33" s="93"/>
-      <c r="B33" s="96"/>
-      <c r="C33" s="67" t="s">
+      <c r="A33" s="88"/>
+      <c r="B33" s="91"/>
+      <c r="C33" s="71" t="s">
         <v>42</v>
       </c>
       <c r="D33" s="40" t="s">
@@ -2454,9 +2471,9 @@
       <c r="M33" s="1"/>
     </row>
     <row r="34" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A34" s="93"/>
-      <c r="B34" s="96"/>
-      <c r="C34" s="67"/>
+      <c r="A34" s="88"/>
+      <c r="B34" s="91"/>
+      <c r="C34" s="71"/>
       <c r="D34" s="28" t="s">
         <v>149</v>
       </c>
@@ -2471,9 +2488,9 @@
       <c r="M34" s="1"/>
     </row>
     <row r="35" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A35" s="93"/>
-      <c r="B35" s="96"/>
-      <c r="C35" s="67" t="s">
+      <c r="A35" s="88"/>
+      <c r="B35" s="91"/>
+      <c r="C35" s="71" t="s">
         <v>43</v>
       </c>
       <c r="D35" s="40" t="s">
@@ -2490,9 +2507,9 @@
       <c r="M35" s="1"/>
     </row>
     <row r="36" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A36" s="93"/>
-      <c r="B36" s="96"/>
-      <c r="C36" s="67"/>
+      <c r="A36" s="88"/>
+      <c r="B36" s="91"/>
+      <c r="C36" s="71"/>
       <c r="D36" s="28" t="s">
         <v>149</v>
       </c>
@@ -2507,8 +2524,8 @@
       <c r="M36" s="1"/>
     </row>
     <row r="37" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A37" s="93"/>
-      <c r="B37" s="96"/>
+      <c r="A37" s="88"/>
+      <c r="B37" s="91"/>
       <c r="C37" s="7" t="s">
         <v>44</v>
       </c>
@@ -2526,9 +2543,9 @@
       <c r="M37" s="1"/>
     </row>
     <row r="38" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A38" s="93"/>
-      <c r="B38" s="96"/>
-      <c r="C38" s="67" t="s">
+      <c r="A38" s="88"/>
+      <c r="B38" s="91"/>
+      <c r="C38" s="71" t="s">
         <v>45</v>
       </c>
       <c r="D38" s="41" t="s">
@@ -2545,9 +2562,9 @@
       <c r="M38" s="1"/>
     </row>
     <row r="39" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A39" s="93"/>
-      <c r="B39" s="96"/>
-      <c r="C39" s="67"/>
+      <c r="A39" s="88"/>
+      <c r="B39" s="91"/>
+      <c r="C39" s="71"/>
       <c r="D39" s="41" t="s">
         <v>148</v>
       </c>
@@ -2562,9 +2579,9 @@
       <c r="M39" s="1"/>
     </row>
     <row r="40" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A40" s="93"/>
-      <c r="B40" s="96"/>
-      <c r="C40" s="67"/>
+      <c r="A40" s="88"/>
+      <c r="B40" s="91"/>
+      <c r="C40" s="71"/>
       <c r="D40" s="28" t="s">
         <v>149</v>
       </c>
@@ -2579,9 +2596,9 @@
       <c r="M40" s="1"/>
     </row>
     <row r="41" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A41" s="93"/>
-      <c r="B41" s="96"/>
-      <c r="C41" s="67" t="s">
+      <c r="A41" s="88"/>
+      <c r="B41" s="91"/>
+      <c r="C41" s="71" t="s">
         <v>46</v>
       </c>
       <c r="D41" s="16" t="s">
@@ -2598,9 +2615,9 @@
       <c r="M41" s="1"/>
     </row>
     <row r="42" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A42" s="93"/>
-      <c r="B42" s="96"/>
-      <c r="C42" s="67"/>
+      <c r="A42" s="88"/>
+      <c r="B42" s="91"/>
+      <c r="C42" s="71"/>
       <c r="D42" s="28" t="s">
         <v>149</v>
       </c>
@@ -2615,8 +2632,8 @@
       <c r="M42" s="1"/>
     </row>
     <row r="43" spans="1:13" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A43" s="93"/>
-      <c r="B43" s="96"/>
+      <c r="A43" s="88"/>
+      <c r="B43" s="91"/>
       <c r="C43" s="57" t="s">
         <v>215</v>
       </c>
@@ -2634,8 +2651,8 @@
       <c r="M43" s="1"/>
     </row>
     <row r="44" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A44" s="93"/>
-      <c r="B44" s="96"/>
+      <c r="A44" s="88"/>
+      <c r="B44" s="91"/>
       <c r="C44" s="7" t="s">
         <v>47</v>
       </c>
@@ -2653,9 +2670,9 @@
       <c r="M44" s="1"/>
     </row>
     <row r="45" spans="1:13" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="A45" s="93"/>
-      <c r="B45" s="96"/>
-      <c r="C45" s="67" t="s">
+      <c r="A45" s="88"/>
+      <c r="B45" s="91"/>
+      <c r="C45" s="71" t="s">
         <v>48</v>
       </c>
       <c r="D45" s="39" t="s">
@@ -2672,9 +2689,9 @@
       <c r="M45" s="1"/>
     </row>
     <row r="46" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A46" s="93"/>
-      <c r="B46" s="96"/>
-      <c r="C46" s="67"/>
+      <c r="A46" s="88"/>
+      <c r="B46" s="91"/>
+      <c r="C46" s="71"/>
       <c r="D46" s="26" t="s">
         <v>8</v>
       </c>
@@ -2689,9 +2706,9 @@
       <c r="M46" s="1"/>
     </row>
     <row r="47" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A47" s="93"/>
-      <c r="B47" s="96"/>
-      <c r="C47" s="67" t="s">
+      <c r="A47" s="88"/>
+      <c r="B47" s="91"/>
+      <c r="C47" s="71" t="s">
         <v>49</v>
       </c>
       <c r="D47" s="26" t="s">
@@ -2708,9 +2725,9 @@
       <c r="M47" s="1"/>
     </row>
     <row r="48" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A48" s="93"/>
-      <c r="B48" s="96"/>
-      <c r="C48" s="67"/>
+      <c r="A48" s="88"/>
+      <c r="B48" s="91"/>
+      <c r="C48" s="71"/>
       <c r="D48" s="26" t="s">
         <v>8</v>
       </c>
@@ -2725,9 +2742,9 @@
       <c r="M48" s="1"/>
     </row>
     <row r="49" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A49" s="93"/>
-      <c r="B49" s="96"/>
-      <c r="C49" s="67" t="s">
+      <c r="A49" s="88"/>
+      <c r="B49" s="91"/>
+      <c r="C49" s="71" t="s">
         <v>50</v>
       </c>
       <c r="D49" s="26" t="s">
@@ -2744,9 +2761,9 @@
       <c r="M49" s="1"/>
     </row>
     <row r="50" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A50" s="93"/>
-      <c r="B50" s="96"/>
-      <c r="C50" s="67"/>
+      <c r="A50" s="88"/>
+      <c r="B50" s="91"/>
+      <c r="C50" s="71"/>
       <c r="D50" s="26" t="s">
         <v>8</v>
       </c>
@@ -2761,9 +2778,9 @@
       <c r="M50" s="1"/>
     </row>
     <row r="51" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A51" s="93"/>
-      <c r="B51" s="96"/>
-      <c r="C51" s="67" t="s">
+      <c r="A51" s="88"/>
+      <c r="B51" s="91"/>
+      <c r="C51" s="71" t="s">
         <v>51</v>
       </c>
       <c r="D51" s="26" t="s">
@@ -2780,9 +2797,9 @@
       <c r="M51" s="1"/>
     </row>
     <row r="52" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A52" s="93"/>
-      <c r="B52" s="96"/>
-      <c r="C52" s="67"/>
+      <c r="A52" s="88"/>
+      <c r="B52" s="91"/>
+      <c r="C52" s="71"/>
       <c r="D52" s="26" t="s">
         <v>8</v>
       </c>
@@ -2797,9 +2814,9 @@
       <c r="M52" s="1"/>
     </row>
     <row r="53" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A53" s="93"/>
-      <c r="B53" s="96"/>
-      <c r="C53" s="67" t="s">
+      <c r="A53" s="88"/>
+      <c r="B53" s="91"/>
+      <c r="C53" s="71" t="s">
         <v>52</v>
       </c>
       <c r="D53" s="26" t="s">
@@ -2816,9 +2833,9 @@
       <c r="M53" s="1"/>
     </row>
     <row r="54" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A54" s="93"/>
-      <c r="B54" s="96"/>
-      <c r="C54" s="67"/>
+      <c r="A54" s="88"/>
+      <c r="B54" s="91"/>
+      <c r="C54" s="71"/>
       <c r="D54" s="26" t="s">
         <v>8</v>
       </c>
@@ -2833,9 +2850,9 @@
       <c r="M54" s="1"/>
     </row>
     <row r="55" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A55" s="93"/>
-      <c r="B55" s="96"/>
-      <c r="C55" s="67" t="s">
+      <c r="A55" s="88"/>
+      <c r="B55" s="91"/>
+      <c r="C55" s="71" t="s">
         <v>53</v>
       </c>
       <c r="D55" s="26" t="s">
@@ -2852,9 +2869,9 @@
       <c r="M55" s="1"/>
     </row>
     <row r="56" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A56" s="93"/>
-      <c r="B56" s="96"/>
-      <c r="C56" s="67"/>
+      <c r="A56" s="88"/>
+      <c r="B56" s="91"/>
+      <c r="C56" s="71"/>
       <c r="D56" s="26" t="s">
         <v>8</v>
       </c>
@@ -2869,9 +2886,9 @@
       <c r="M56" s="1"/>
     </row>
     <row r="57" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A57" s="93"/>
-      <c r="B57" s="96"/>
-      <c r="C57" s="67" t="s">
+      <c r="A57" s="88"/>
+      <c r="B57" s="91"/>
+      <c r="C57" s="71" t="s">
         <v>54</v>
       </c>
       <c r="D57" s="26" t="s">
@@ -2888,9 +2905,9 @@
       <c r="M57" s="1"/>
     </row>
     <row r="58" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="94"/>
-      <c r="B58" s="86"/>
-      <c r="C58" s="62"/>
+      <c r="A58" s="89"/>
+      <c r="B58" s="92"/>
+      <c r="C58" s="72"/>
       <c r="D58" s="30" t="s">
         <v>8</v>
       </c>
@@ -2905,10 +2922,10 @@
       <c r="M58" s="1"/>
     </row>
     <row r="59" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A59" s="80" t="s">
+      <c r="A59" s="93" t="s">
         <v>55</v>
       </c>
-      <c r="B59" s="83" t="s">
+      <c r="B59" s="73" t="s">
         <v>56</v>
       </c>
       <c r="C59" s="6" t="s">
@@ -2928,9 +2945,9 @@
       <c r="M59" s="1"/>
     </row>
     <row r="60" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A60" s="81"/>
-      <c r="B60" s="84"/>
-      <c r="C60" s="67" t="s">
+      <c r="A60" s="94"/>
+      <c r="B60" s="74"/>
+      <c r="C60" s="71" t="s">
         <v>57</v>
       </c>
       <c r="D60" s="26" t="s">
@@ -2947,9 +2964,9 @@
       <c r="M60" s="1"/>
     </row>
     <row r="61" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A61" s="81"/>
-      <c r="B61" s="84"/>
-      <c r="C61" s="67"/>
+      <c r="A61" s="94"/>
+      <c r="B61" s="74"/>
+      <c r="C61" s="71"/>
       <c r="D61" s="26" t="s">
         <v>8</v>
       </c>
@@ -2964,9 +2981,9 @@
       <c r="M61" s="1"/>
     </row>
     <row r="62" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A62" s="81"/>
-      <c r="B62" s="84"/>
-      <c r="C62" s="67" t="s">
+      <c r="A62" s="94"/>
+      <c r="B62" s="74"/>
+      <c r="C62" s="71" t="s">
         <v>59</v>
       </c>
       <c r="D62" s="26" t="s">
@@ -2983,9 +3000,9 @@
       <c r="M62" s="1"/>
     </row>
     <row r="63" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A63" s="81"/>
-      <c r="B63" s="84"/>
-      <c r="C63" s="67"/>
+      <c r="A63" s="94"/>
+      <c r="B63" s="74"/>
+      <c r="C63" s="71"/>
       <c r="D63" s="26" t="s">
         <v>8</v>
       </c>
@@ -3000,9 +3017,9 @@
       <c r="M63" s="1"/>
     </row>
     <row r="64" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A64" s="81"/>
-      <c r="B64" s="84"/>
-      <c r="C64" s="67" t="s">
+      <c r="A64" s="94"/>
+      <c r="B64" s="74"/>
+      <c r="C64" s="71" t="s">
         <v>60</v>
       </c>
       <c r="D64" s="26" t="s">
@@ -3019,9 +3036,9 @@
       <c r="M64" s="1"/>
     </row>
     <row r="65" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A65" s="81"/>
-      <c r="B65" s="84"/>
-      <c r="C65" s="67"/>
+      <c r="A65" s="94"/>
+      <c r="B65" s="74"/>
+      <c r="C65" s="71"/>
       <c r="D65" s="28" t="s">
         <v>149</v>
       </c>
@@ -3036,8 +3053,8 @@
       <c r="M65" s="1"/>
     </row>
     <row r="66" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A66" s="81"/>
-      <c r="B66" s="84"/>
+      <c r="A66" s="94"/>
+      <c r="B66" s="74"/>
       <c r="C66" s="23" t="s">
         <v>61</v>
       </c>
@@ -3055,8 +3072,8 @@
       <c r="M66" s="1"/>
     </row>
     <row r="67" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A67" s="81"/>
-      <c r="B67" s="84"/>
+      <c r="A67" s="94"/>
+      <c r="B67" s="74"/>
       <c r="C67" s="37" t="s">
         <v>158</v>
       </c>
@@ -3074,8 +3091,8 @@
       <c r="M67" s="1"/>
     </row>
     <row r="68" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A68" s="81"/>
-      <c r="B68" s="84"/>
+      <c r="A68" s="94"/>
+      <c r="B68" s="74"/>
       <c r="C68" s="37" t="s">
         <v>159</v>
       </c>
@@ -3093,8 +3110,8 @@
       <c r="M68" s="1"/>
     </row>
     <row r="69" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A69" s="81"/>
-      <c r="B69" s="84"/>
+      <c r="A69" s="94"/>
+      <c r="B69" s="74"/>
       <c r="C69" s="37" t="s">
         <v>160</v>
       </c>
@@ -3112,8 +3129,8 @@
       <c r="M69" s="1"/>
     </row>
     <row r="70" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A70" s="81"/>
-      <c r="B70" s="84"/>
+      <c r="A70" s="94"/>
+      <c r="B70" s="74"/>
       <c r="C70" s="37" t="s">
         <v>161</v>
       </c>
@@ -3131,8 +3148,8 @@
       <c r="M70" s="1"/>
     </row>
     <row r="71" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A71" s="81"/>
-      <c r="B71" s="84"/>
+      <c r="A71" s="94"/>
+      <c r="B71" s="74"/>
       <c r="C71" s="37" t="s">
         <v>162</v>
       </c>
@@ -3150,8 +3167,8 @@
       <c r="M71" s="1"/>
     </row>
     <row r="72" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A72" s="81"/>
-      <c r="B72" s="84"/>
+      <c r="A72" s="94"/>
+      <c r="B72" s="74"/>
       <c r="C72" s="37" t="s">
         <v>163</v>
       </c>
@@ -3169,8 +3186,8 @@
       <c r="M72" s="1"/>
     </row>
     <row r="73" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="81"/>
-      <c r="B73" s="84"/>
+      <c r="A73" s="94"/>
+      <c r="B73" s="74"/>
       <c r="C73" s="38" t="s">
         <v>111</v>
       </c>
@@ -3188,18 +3205,10 @@
       <c r="M73" s="1"/>
     </row>
     <row r="74" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="20" t="s">
-        <v>62</v>
-      </c>
-      <c r="B74" s="21" t="s">
-        <v>63</v>
-      </c>
-      <c r="C74" s="21" t="s">
-        <v>64</v>
-      </c>
-      <c r="D74" s="39" t="s">
-        <v>164</v>
-      </c>
+      <c r="A74" s="61"/>
+      <c r="B74" s="62"/>
+      <c r="C74" s="116"/>
+      <c r="D74" s="39"/>
       <c r="E74" s="60"/>
       <c r="F74" s="1"/>
       <c r="G74" s="1"/>
@@ -3212,20 +3221,24 @@
     </row>
     <row r="75" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="20" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B75" s="21" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C75" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="D75" s="36" t="s">
-        <v>67</v>
+        <v>64</v>
+      </c>
+      <c r="D75" s="39" t="s">
+        <v>164</v>
       </c>
       <c r="E75" s="60"/>
-      <c r="F75" s="1"/>
-      <c r="G75" s="1"/>
+      <c r="F75" s="117" t="s">
+        <v>64</v>
+      </c>
+      <c r="G75" s="118" t="s">
+        <v>164</v>
+      </c>
       <c r="H75" s="1"/>
       <c r="I75" s="1"/>
       <c r="J75" s="1"/>
@@ -3233,18 +3246,18 @@
       <c r="L75" s="1"/>
       <c r="M75" s="1"/>
     </row>
-    <row r="76" spans="1:13" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="A76" s="89" t="s">
-        <v>68</v>
-      </c>
-      <c r="B76" s="61" t="s">
-        <v>69</v>
-      </c>
-      <c r="C76" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="D76" s="45" t="s">
-        <v>165</v>
+    <row r="76" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="B76" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="C76" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="D76" s="36" t="s">
+        <v>67</v>
       </c>
       <c r="E76" s="60"/>
       <c r="F76" s="1"/>
@@ -3256,14 +3269,18 @@
       <c r="L76" s="1"/>
       <c r="M76" s="1"/>
     </row>
-    <row r="77" spans="1:13" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="91"/>
-      <c r="B77" s="68"/>
-      <c r="C77" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="D77" s="30" t="s">
-        <v>166</v>
+    <row r="77" spans="1:13" ht="26.25" x14ac:dyDescent="0.25">
+      <c r="A77" s="67" t="s">
+        <v>68</v>
+      </c>
+      <c r="B77" s="70" t="s">
+        <v>69</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="D77" s="45" t="s">
+        <v>165</v>
       </c>
       <c r="E77" s="60"/>
       <c r="F77" s="1"/>
@@ -3275,18 +3292,14 @@
       <c r="L77" s="1"/>
       <c r="M77" s="1"/>
     </row>
-    <row r="78" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="20" t="s">
-        <v>72</v>
-      </c>
-      <c r="B78" s="21" t="s">
-        <v>73</v>
-      </c>
-      <c r="C78" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="D78" s="29" t="s">
-        <v>67</v>
+    <row r="78" spans="1:13" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="95"/>
+      <c r="B78" s="96"/>
+      <c r="C78" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="D78" s="30" t="s">
+        <v>166</v>
       </c>
       <c r="E78" s="60"/>
       <c r="F78" s="1"/>
@@ -3300,10 +3313,10 @@
     </row>
     <row r="79" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="20" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B79" s="21" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C79" s="21" t="s">
         <v>67</v>
@@ -3321,18 +3334,18 @@
       <c r="L79" s="1"/>
       <c r="M79" s="1"/>
     </row>
-    <row r="80" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A80" s="80" t="s">
-        <v>76</v>
-      </c>
-      <c r="B80" s="83" t="s">
-        <v>77</v>
-      </c>
-      <c r="C80" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="D80" s="25" t="s">
-        <v>167</v>
+    <row r="80" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="20" t="s">
+        <v>74</v>
+      </c>
+      <c r="B80" s="21" t="s">
+        <v>75</v>
+      </c>
+      <c r="C80" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="D80" s="29" t="s">
+        <v>67</v>
       </c>
       <c r="E80" s="60"/>
       <c r="F80" s="1"/>
@@ -3345,13 +3358,17 @@
       <c r="M80" s="1"/>
     </row>
     <row r="81" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A81" s="81"/>
-      <c r="B81" s="84"/>
-      <c r="C81" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="D81" s="26" t="s">
-        <v>168</v>
+      <c r="A81" s="93" t="s">
+        <v>76</v>
+      </c>
+      <c r="B81" s="73" t="s">
+        <v>77</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="D81" s="25" t="s">
+        <v>167</v>
       </c>
       <c r="E81" s="60"/>
       <c r="F81" s="1"/>
@@ -3364,10 +3381,10 @@
       <c r="M81" s="1"/>
     </row>
     <row r="82" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A82" s="81"/>
-      <c r="B82" s="84"/>
+      <c r="A82" s="94"/>
+      <c r="B82" s="74"/>
       <c r="C82" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D82" s="26" t="s">
         <v>168</v>
@@ -3383,13 +3400,13 @@
       <c r="M82" s="1"/>
     </row>
     <row r="83" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A83" s="81"/>
-      <c r="B83" s="84"/>
+      <c r="A83" s="94"/>
+      <c r="B83" s="74"/>
       <c r="C83" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D83" s="26" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E83" s="60"/>
       <c r="F83" s="1"/>
@@ -3402,13 +3419,13 @@
       <c r="M83" s="1"/>
     </row>
     <row r="84" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A84" s="81"/>
-      <c r="B84" s="84"/>
+      <c r="A84" s="94"/>
+      <c r="B84" s="74"/>
       <c r="C84" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D84" s="26" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E84" s="60"/>
       <c r="F84" s="1"/>
@@ -3421,13 +3438,13 @@
       <c r="M84" s="1"/>
     </row>
     <row r="85" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A85" s="81"/>
-      <c r="B85" s="84"/>
+      <c r="A85" s="94"/>
+      <c r="B85" s="74"/>
       <c r="C85" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="D85" s="40" t="s">
-        <v>171</v>
+        <v>82</v>
+      </c>
+      <c r="D85" s="26" t="s">
+        <v>170</v>
       </c>
       <c r="E85" s="60"/>
       <c r="F85" s="1"/>
@@ -3440,13 +3457,13 @@
       <c r="M85" s="1"/>
     </row>
     <row r="86" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A86" s="81"/>
-      <c r="B86" s="84"/>
+      <c r="A86" s="94"/>
+      <c r="B86" s="74"/>
       <c r="C86" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="D86" s="41" t="s">
-        <v>172</v>
+        <v>83</v>
+      </c>
+      <c r="D86" s="40" t="s">
+        <v>171</v>
       </c>
       <c r="E86" s="60"/>
       <c r="F86" s="1"/>
@@ -3459,18 +3476,16 @@
       <c r="M86" s="1"/>
     </row>
     <row r="87" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A87" s="81"/>
-      <c r="B87" s="84"/>
-      <c r="C87" s="67" t="s">
-        <v>85</v>
-      </c>
-      <c r="D87" s="26" t="s">
-        <v>173</v>
-      </c>
-      <c r="E87" s="110"/>
-      <c r="F87" s="1" t="s">
-        <v>218</v>
-      </c>
+      <c r="A87" s="94"/>
+      <c r="B87" s="74"/>
+      <c r="C87" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="D87" s="41" t="s">
+        <v>172</v>
+      </c>
+      <c r="E87" s="60"/>
+      <c r="F87" s="1"/>
       <c r="G87" s="1"/>
       <c r="H87" s="1"/>
       <c r="I87" s="1"/>
@@ -3479,15 +3494,19 @@
       <c r="L87" s="1"/>
       <c r="M87" s="1"/>
     </row>
-    <row r="88" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="82"/>
-      <c r="B88" s="85"/>
-      <c r="C88" s="68"/>
-      <c r="D88" s="30" t="s">
-        <v>8</v>
-      </c>
-      <c r="E88" s="110"/>
-      <c r="F88" s="1"/>
+    <row r="88" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A88" s="94"/>
+      <c r="B88" s="74"/>
+      <c r="C88" s="71" t="s">
+        <v>85</v>
+      </c>
+      <c r="D88" s="26" t="s">
+        <v>173</v>
+      </c>
+      <c r="E88" s="65"/>
+      <c r="F88" s="1" t="s">
+        <v>218</v>
+      </c>
       <c r="G88" s="1"/>
       <c r="H88" s="1"/>
       <c r="I88" s="1"/>
@@ -3496,20 +3515,14 @@
       <c r="L88" s="1"/>
       <c r="M88" s="1"/>
     </row>
-    <row r="89" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A89" s="80" t="s">
-        <v>86</v>
-      </c>
-      <c r="B89" s="83" t="s">
-        <v>87</v>
-      </c>
-      <c r="C89" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="D89" s="25" t="s">
-        <v>174</v>
-      </c>
-      <c r="E89" s="60"/>
+    <row r="89" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="97"/>
+      <c r="B89" s="75"/>
+      <c r="C89" s="96"/>
+      <c r="D89" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="E89" s="59"/>
       <c r="F89" s="1"/>
       <c r="G89" s="1"/>
       <c r="H89" s="1"/>
@@ -3519,14 +3532,18 @@
       <c r="L89" s="1"/>
       <c r="M89" s="1"/>
     </row>
-    <row r="90" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="81"/>
-      <c r="B90" s="84"/>
-      <c r="C90" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="D90" s="27" t="s">
-        <v>175</v>
+    <row r="90" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A90" s="93" t="s">
+        <v>86</v>
+      </c>
+      <c r="B90" s="73" t="s">
+        <v>87</v>
+      </c>
+      <c r="C90" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D90" s="25" t="s">
+        <v>174</v>
       </c>
       <c r="E90" s="60"/>
       <c r="F90" s="1"/>
@@ -3538,18 +3555,14 @@
       <c r="L90" s="1"/>
       <c r="M90" s="1"/>
     </row>
-    <row r="91" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A91" s="89" t="s">
-        <v>90</v>
-      </c>
-      <c r="B91" s="61" t="s">
-        <v>91</v>
-      </c>
-      <c r="C91" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="D91" s="25" t="s">
-        <v>176</v>
+    <row r="91" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A91" s="94"/>
+      <c r="B91" s="74"/>
+      <c r="C91" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="D91" s="27" t="s">
+        <v>175</v>
       </c>
       <c r="E91" s="60"/>
       <c r="F91" s="1"/>
@@ -3562,13 +3575,17 @@
       <c r="M91" s="1"/>
     </row>
     <row r="92" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A92" s="90"/>
-      <c r="B92" s="67"/>
-      <c r="C92" s="67" t="s">
-        <v>93</v>
-      </c>
-      <c r="D92" s="26" t="s">
-        <v>177</v>
+      <c r="A92" s="67" t="s">
+        <v>90</v>
+      </c>
+      <c r="B92" s="70" t="s">
+        <v>91</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="D92" s="25" t="s">
+        <v>176</v>
       </c>
       <c r="E92" s="60"/>
       <c r="F92" s="1"/>
@@ -3581,13 +3598,15 @@
       <c r="M92" s="1"/>
     </row>
     <row r="93" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A93" s="90"/>
-      <c r="B93" s="67"/>
-      <c r="C93" s="67"/>
+      <c r="A93" s="68"/>
+      <c r="B93" s="71"/>
+      <c r="C93" s="71" t="s">
+        <v>93</v>
+      </c>
       <c r="D93" s="26" t="s">
-        <v>8</v>
-      </c>
-      <c r="E93" s="111"/>
+        <v>177</v>
+      </c>
+      <c r="E93" s="63"/>
       <c r="F93" s="1"/>
       <c r="G93" s="1"/>
       <c r="H93" s="1"/>
@@ -3598,15 +3617,13 @@
       <c r="M93" s="1"/>
     </row>
     <row r="94" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A94" s="90"/>
-      <c r="B94" s="67"/>
-      <c r="C94" s="67" t="s">
-        <v>94</v>
-      </c>
+      <c r="A94" s="68"/>
+      <c r="B94" s="71"/>
+      <c r="C94" s="71"/>
       <c r="D94" s="26" t="s">
-        <v>178</v>
-      </c>
-      <c r="E94" s="111"/>
+        <v>8</v>
+      </c>
+      <c r="E94" s="63"/>
       <c r="F94" s="1"/>
       <c r="G94" s="1"/>
       <c r="H94" s="1"/>
@@ -3617,13 +3634,15 @@
       <c r="M94" s="1"/>
     </row>
     <row r="95" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A95" s="90"/>
-      <c r="B95" s="67"/>
-      <c r="C95" s="67"/>
+      <c r="A95" s="68"/>
+      <c r="B95" s="71"/>
+      <c r="C95" s="71" t="s">
+        <v>94</v>
+      </c>
       <c r="D95" s="26" t="s">
-        <v>8</v>
-      </c>
-      <c r="E95" s="111"/>
+        <v>178</v>
+      </c>
+      <c r="E95" s="63"/>
       <c r="F95" s="1"/>
       <c r="G95" s="1"/>
       <c r="H95" s="1"/>
@@ -3634,15 +3653,13 @@
       <c r="M95" s="1"/>
     </row>
     <row r="96" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A96" s="90"/>
-      <c r="B96" s="67"/>
-      <c r="C96" s="67" t="s">
-        <v>95</v>
-      </c>
+      <c r="A96" s="68"/>
+      <c r="B96" s="71"/>
+      <c r="C96" s="71"/>
       <c r="D96" s="26" t="s">
-        <v>179</v>
-      </c>
-      <c r="E96" s="60"/>
+        <v>8</v>
+      </c>
+      <c r="E96" s="63"/>
       <c r="F96" s="1"/>
       <c r="G96" s="1"/>
       <c r="H96" s="1"/>
@@ -3652,12 +3669,14 @@
       <c r="L96" s="1"/>
       <c r="M96" s="1"/>
     </row>
-    <row r="97" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A97" s="91"/>
-      <c r="B97" s="68"/>
-      <c r="C97" s="68"/>
-      <c r="D97" s="30" t="s">
-        <v>8</v>
+    <row r="97" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A97" s="68"/>
+      <c r="B97" s="71"/>
+      <c r="C97" s="71" t="s">
+        <v>95</v>
+      </c>
+      <c r="D97" s="26" t="s">
+        <v>179</v>
       </c>
       <c r="E97" s="60"/>
       <c r="F97" s="1"/>
@@ -3669,18 +3688,12 @@
       <c r="L97" s="1"/>
       <c r="M97" s="1"/>
     </row>
-    <row r="98" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A98" s="80" t="s">
-        <v>96</v>
-      </c>
-      <c r="B98" s="83" t="s">
-        <v>97</v>
-      </c>
-      <c r="C98" s="83" t="s">
-        <v>184</v>
-      </c>
-      <c r="D98" s="25" t="s">
-        <v>183</v>
+    <row r="98" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A98" s="95"/>
+      <c r="B98" s="96"/>
+      <c r="C98" s="96"/>
+      <c r="D98" s="30" t="s">
+        <v>8</v>
       </c>
       <c r="E98" s="60"/>
       <c r="F98" s="1"/>
@@ -3693,11 +3706,17 @@
       <c r="M98" s="1"/>
     </row>
     <row r="99" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A99" s="81"/>
-      <c r="B99" s="84"/>
-      <c r="C99" s="79"/>
-      <c r="D99" s="46" t="s">
-        <v>8</v>
+      <c r="A99" s="93" t="s">
+        <v>96</v>
+      </c>
+      <c r="B99" s="73" t="s">
+        <v>97</v>
+      </c>
+      <c r="C99" s="73" t="s">
+        <v>184</v>
+      </c>
+      <c r="D99" s="25" t="s">
+        <v>183</v>
       </c>
       <c r="E99" s="60"/>
       <c r="F99" s="1"/>
@@ -3710,13 +3729,11 @@
       <c r="M99" s="1"/>
     </row>
     <row r="100" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A100" s="81"/>
-      <c r="B100" s="84"/>
-      <c r="C100" s="62" t="s">
-        <v>185</v>
-      </c>
+      <c r="A100" s="94"/>
+      <c r="B100" s="74"/>
+      <c r="C100" s="98"/>
       <c r="D100" s="46" t="s">
-        <v>183</v>
+        <v>8</v>
       </c>
       <c r="E100" s="60"/>
       <c r="F100" s="1"/>
@@ -3729,11 +3746,13 @@
       <c r="M100" s="1"/>
     </row>
     <row r="101" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A101" s="81"/>
-      <c r="B101" s="84"/>
-      <c r="C101" s="79"/>
+      <c r="A101" s="94"/>
+      <c r="B101" s="74"/>
+      <c r="C101" s="72" t="s">
+        <v>185</v>
+      </c>
       <c r="D101" s="46" t="s">
-        <v>8</v>
+        <v>183</v>
       </c>
       <c r="E101" s="60"/>
       <c r="F101" s="1"/>
@@ -3746,13 +3765,11 @@
       <c r="M101" s="1"/>
     </row>
     <row r="102" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A102" s="81"/>
-      <c r="B102" s="84"/>
-      <c r="C102" s="62" t="s">
-        <v>186</v>
-      </c>
+      <c r="A102" s="94"/>
+      <c r="B102" s="74"/>
+      <c r="C102" s="98"/>
       <c r="D102" s="46" t="s">
-        <v>183</v>
+        <v>8</v>
       </c>
       <c r="E102" s="60"/>
       <c r="F102" s="1"/>
@@ -3765,11 +3782,13 @@
       <c r="M102" s="1"/>
     </row>
     <row r="103" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A103" s="81"/>
-      <c r="B103" s="84"/>
-      <c r="C103" s="79"/>
+      <c r="A103" s="94"/>
+      <c r="B103" s="74"/>
+      <c r="C103" s="72" t="s">
+        <v>186</v>
+      </c>
       <c r="D103" s="46" t="s">
-        <v>8</v>
+        <v>183</v>
       </c>
       <c r="E103" s="60"/>
       <c r="F103" s="1"/>
@@ -3782,13 +3801,11 @@
       <c r="M103" s="1"/>
     </row>
     <row r="104" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A104" s="81"/>
-      <c r="B104" s="84"/>
-      <c r="C104" s="62" t="s">
-        <v>187</v>
-      </c>
+      <c r="A104" s="94"/>
+      <c r="B104" s="74"/>
+      <c r="C104" s="98"/>
       <c r="D104" s="46" t="s">
-        <v>183</v>
+        <v>8</v>
       </c>
       <c r="E104" s="60"/>
       <c r="F104" s="1"/>
@@ -3801,11 +3818,13 @@
       <c r="M104" s="1"/>
     </row>
     <row r="105" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A105" s="81"/>
-      <c r="B105" s="84"/>
-      <c r="C105" s="79"/>
+      <c r="A105" s="94"/>
+      <c r="B105" s="74"/>
+      <c r="C105" s="72" t="s">
+        <v>187</v>
+      </c>
       <c r="D105" s="46" t="s">
-        <v>8</v>
+        <v>183</v>
       </c>
       <c r="E105" s="60"/>
       <c r="F105" s="1"/>
@@ -3818,13 +3837,11 @@
       <c r="M105" s="1"/>
     </row>
     <row r="106" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A106" s="81"/>
-      <c r="B106" s="84"/>
-      <c r="C106" s="62" t="s">
-        <v>98</v>
-      </c>
+      <c r="A106" s="94"/>
+      <c r="B106" s="74"/>
+      <c r="C106" s="98"/>
       <c r="D106" s="46" t="s">
-        <v>180</v>
+        <v>8</v>
       </c>
       <c r="E106" s="60"/>
       <c r="F106" s="1"/>
@@ -3837,11 +3854,13 @@
       <c r="M106" s="1"/>
     </row>
     <row r="107" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A107" s="81"/>
-      <c r="B107" s="84"/>
-      <c r="C107" s="79"/>
-      <c r="D107" s="26" t="s">
-        <v>183</v>
+      <c r="A107" s="94"/>
+      <c r="B107" s="74"/>
+      <c r="C107" s="72" t="s">
+        <v>98</v>
+      </c>
+      <c r="D107" s="46" t="s">
+        <v>180</v>
       </c>
       <c r="E107" s="60"/>
       <c r="F107" s="1"/>
@@ -3853,14 +3872,12 @@
       <c r="L107" s="1"/>
       <c r="M107" s="1"/>
     </row>
-    <row r="108" spans="1:13" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="A108" s="81"/>
-      <c r="B108" s="84"/>
-      <c r="C108" s="62" t="s">
-        <v>99</v>
-      </c>
+    <row r="108" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A108" s="94"/>
+      <c r="B108" s="74"/>
+      <c r="C108" s="98"/>
       <c r="D108" s="26" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="E108" s="60"/>
       <c r="F108" s="1"/>
@@ -3872,12 +3889,14 @@
       <c r="L108" s="1"/>
       <c r="M108" s="1"/>
     </row>
-    <row r="109" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A109" s="81"/>
-      <c r="B109" s="84"/>
-      <c r="C109" s="79"/>
+    <row r="109" spans="1:13" ht="26.25" x14ac:dyDescent="0.25">
+      <c r="A109" s="94"/>
+      <c r="B109" s="74"/>
+      <c r="C109" s="72" t="s">
+        <v>99</v>
+      </c>
       <c r="D109" s="26" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="E109" s="60"/>
       <c r="F109" s="1"/>
@@ -3890,11 +3909,9 @@
       <c r="M109" s="1"/>
     </row>
     <row r="110" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A110" s="81"/>
-      <c r="B110" s="84"/>
-      <c r="C110" s="62" t="s">
-        <v>188</v>
-      </c>
+      <c r="A110" s="94"/>
+      <c r="B110" s="74"/>
+      <c r="C110" s="98"/>
       <c r="D110" s="26" t="s">
         <v>183</v>
       </c>
@@ -3909,11 +3926,13 @@
       <c r="M110" s="1"/>
     </row>
     <row r="111" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A111" s="81"/>
-      <c r="B111" s="84"/>
-      <c r="C111" s="79"/>
+      <c r="A111" s="94"/>
+      <c r="B111" s="74"/>
+      <c r="C111" s="72" t="s">
+        <v>188</v>
+      </c>
       <c r="D111" s="26" t="s">
-        <v>8</v>
+        <v>183</v>
       </c>
       <c r="E111" s="60"/>
       <c r="F111" s="1"/>
@@ -3926,13 +3945,11 @@
       <c r="M111" s="1"/>
     </row>
     <row r="112" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A112" s="81"/>
-      <c r="B112" s="84"/>
-      <c r="C112" s="62" t="s">
-        <v>189</v>
-      </c>
+      <c r="A112" s="94"/>
+      <c r="B112" s="74"/>
+      <c r="C112" s="98"/>
       <c r="D112" s="26" t="s">
-        <v>183</v>
+        <v>8</v>
       </c>
       <c r="E112" s="60"/>
       <c r="F112" s="1"/>
@@ -3945,11 +3962,13 @@
       <c r="M112" s="1"/>
     </row>
     <row r="113" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A113" s="81"/>
-      <c r="B113" s="84"/>
-      <c r="C113" s="79"/>
+      <c r="A113" s="94"/>
+      <c r="B113" s="74"/>
+      <c r="C113" s="72" t="s">
+        <v>189</v>
+      </c>
       <c r="D113" s="26" t="s">
-        <v>8</v>
+        <v>183</v>
       </c>
       <c r="E113" s="60"/>
       <c r="F113" s="1"/>
@@ -3962,13 +3981,11 @@
       <c r="M113" s="1"/>
     </row>
     <row r="114" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A114" s="81"/>
-      <c r="B114" s="84"/>
-      <c r="C114" s="62" t="s">
-        <v>190</v>
-      </c>
+      <c r="A114" s="94"/>
+      <c r="B114" s="74"/>
+      <c r="C114" s="98"/>
       <c r="D114" s="26" t="s">
-        <v>183</v>
+        <v>8</v>
       </c>
       <c r="E114" s="60"/>
       <c r="F114" s="1"/>
@@ -3981,11 +3998,13 @@
       <c r="M114" s="1"/>
     </row>
     <row r="115" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A115" s="81"/>
-      <c r="B115" s="84"/>
-      <c r="C115" s="79"/>
+      <c r="A115" s="94"/>
+      <c r="B115" s="74"/>
+      <c r="C115" s="72" t="s">
+        <v>190</v>
+      </c>
       <c r="D115" s="26" t="s">
-        <v>8</v>
+        <v>183</v>
       </c>
       <c r="E115" s="60"/>
       <c r="F115" s="1"/>
@@ -3998,13 +4017,11 @@
       <c r="M115" s="1"/>
     </row>
     <row r="116" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A116" s="81"/>
-      <c r="B116" s="84"/>
-      <c r="C116" s="62" t="s">
-        <v>191</v>
-      </c>
+      <c r="A116" s="94"/>
+      <c r="B116" s="74"/>
+      <c r="C116" s="98"/>
       <c r="D116" s="26" t="s">
-        <v>183</v>
+        <v>8</v>
       </c>
       <c r="E116" s="60"/>
       <c r="F116" s="1"/>
@@ -4016,12 +4033,14 @@
       <c r="L116" s="1"/>
       <c r="M116" s="1"/>
     </row>
-    <row r="117" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A117" s="82"/>
-      <c r="B117" s="85"/>
-      <c r="C117" s="85"/>
-      <c r="D117" s="30" t="s">
-        <v>8</v>
+    <row r="117" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A117" s="94"/>
+      <c r="B117" s="74"/>
+      <c r="C117" s="72" t="s">
+        <v>191</v>
+      </c>
+      <c r="D117" s="26" t="s">
+        <v>183</v>
       </c>
       <c r="E117" s="60"/>
       <c r="F117" s="1"/>
@@ -4033,20 +4052,14 @@
       <c r="L117" s="1"/>
       <c r="M117" s="1"/>
     </row>
-    <row r="118" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A118" s="80" t="s">
-        <v>101</v>
-      </c>
-      <c r="B118" s="83" t="s">
-        <v>102</v>
-      </c>
-      <c r="C118" s="83" t="s">
-        <v>100</v>
-      </c>
-      <c r="D118" s="47" t="s">
-        <v>213</v>
-      </c>
-      <c r="E118" s="111"/>
+    <row r="118" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A118" s="97"/>
+      <c r="B118" s="75"/>
+      <c r="C118" s="75"/>
+      <c r="D118" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="E118" s="60"/>
       <c r="F118" s="1"/>
       <c r="G118" s="1"/>
       <c r="H118" s="1"/>
@@ -4056,560 +4069,587 @@
       <c r="L118" s="1"/>
       <c r="M118" s="1"/>
     </row>
-    <row r="119" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A119" s="81"/>
-      <c r="B119" s="84"/>
-      <c r="C119" s="84"/>
-      <c r="D119" s="32" t="s">
+    <row r="119" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A119" s="93" t="s">
+        <v>101</v>
+      </c>
+      <c r="B119" s="73" t="s">
+        <v>102</v>
+      </c>
+      <c r="C119" s="73" t="s">
+        <v>100</v>
+      </c>
+      <c r="D119" s="47" t="s">
+        <v>213</v>
+      </c>
+      <c r="E119" s="63"/>
+      <c r="F119" s="1"/>
+      <c r="G119" s="1"/>
+      <c r="H119" s="1"/>
+      <c r="I119" s="1"/>
+      <c r="J119" s="1"/>
+      <c r="K119" s="1"/>
+      <c r="L119" s="1"/>
+      <c r="M119" s="1"/>
+    </row>
+    <row r="120" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A120" s="94"/>
+      <c r="B120" s="74"/>
+      <c r="C120" s="74"/>
+      <c r="D120" s="32" t="s">
         <v>182</v>
       </c>
-      <c r="E119" s="112"/>
-    </row>
-    <row r="120" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A120" s="81"/>
-      <c r="B120" s="84"/>
-      <c r="C120" s="79"/>
-      <c r="D120" s="32" t="s">
+      <c r="E120" s="64"/>
+    </row>
+    <row r="121" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A121" s="94"/>
+      <c r="B121" s="74"/>
+      <c r="C121" s="98"/>
+      <c r="D121" s="32" t="s">
         <v>183</v>
       </c>
-      <c r="E120" s="112"/>
-    </row>
-    <row r="121" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A121" s="81"/>
-      <c r="B121" s="84"/>
-      <c r="C121" s="62" t="s">
+      <c r="E121" s="64"/>
+    </row>
+    <row r="122" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A122" s="94"/>
+      <c r="B122" s="74"/>
+      <c r="C122" s="72" t="s">
         <v>192</v>
       </c>
-      <c r="D121" s="26" t="s">
+      <c r="D122" s="26" t="s">
         <v>183</v>
       </c>
-      <c r="E121" s="113"/>
-    </row>
-    <row r="122" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A122" s="81"/>
-      <c r="B122" s="84"/>
-      <c r="C122" s="79"/>
-      <c r="D122" s="30" t="s">
+      <c r="E122" s="65"/>
+    </row>
+    <row r="123" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A123" s="94"/>
+      <c r="B123" s="74"/>
+      <c r="C123" s="98"/>
+      <c r="D123" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="E122" s="113"/>
-    </row>
-    <row r="123" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A123" s="81"/>
-      <c r="B123" s="84"/>
-      <c r="C123" s="62" t="s">
+      <c r="E123" s="65"/>
+    </row>
+    <row r="124" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A124" s="94"/>
+      <c r="B124" s="74"/>
+      <c r="C124" s="72" t="s">
         <v>193</v>
       </c>
-      <c r="D123" s="26" t="s">
+      <c r="D124" s="26" t="s">
         <v>183</v>
       </c>
-      <c r="E123" s="113"/>
-    </row>
-    <row r="124" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A124" s="81"/>
-      <c r="B124" s="84"/>
-      <c r="C124" s="79"/>
-      <c r="D124" s="30" t="s">
+      <c r="E124" s="65"/>
+    </row>
+    <row r="125" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A125" s="94"/>
+      <c r="B125" s="74"/>
+      <c r="C125" s="98"/>
+      <c r="D125" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="E124" s="113"/>
-    </row>
-    <row r="125" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A125" s="81"/>
-      <c r="B125" s="84"/>
-      <c r="C125" s="62" t="s">
+      <c r="E125" s="65"/>
+    </row>
+    <row r="126" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A126" s="94"/>
+      <c r="B126" s="74"/>
+      <c r="C126" s="72" t="s">
         <v>194</v>
       </c>
-      <c r="D125" s="26" t="s">
+      <c r="D126" s="26" t="s">
         <v>183</v>
       </c>
-      <c r="E125" s="113"/>
-    </row>
-    <row r="126" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A126" s="81"/>
-      <c r="B126" s="84"/>
-      <c r="C126" s="79"/>
-      <c r="D126" s="30" t="s">
+      <c r="E126" s="65"/>
+    </row>
+    <row r="127" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A127" s="94"/>
+      <c r="B127" s="74"/>
+      <c r="C127" s="98"/>
+      <c r="D127" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="E126" s="113"/>
-    </row>
-    <row r="127" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A127" s="81"/>
-      <c r="B127" s="84"/>
-      <c r="C127" s="67" t="s">
+      <c r="E127" s="65"/>
+    </row>
+    <row r="128" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A128" s="94"/>
+      <c r="B128" s="74"/>
+      <c r="C128" s="71" t="s">
         <v>103</v>
       </c>
-      <c r="D127" s="26" t="s">
+      <c r="D128" s="26" t="s">
         <v>214</v>
       </c>
-      <c r="E127" s="114"/>
-    </row>
-    <row r="128" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A128" s="81"/>
-      <c r="B128" s="84"/>
-      <c r="C128" s="67"/>
-      <c r="D128" s="26" t="s">
+      <c r="E128" s="66"/>
+    </row>
+    <row r="129" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A129" s="94"/>
+      <c r="B129" s="74"/>
+      <c r="C129" s="71"/>
+      <c r="D129" s="26" t="s">
         <v>183</v>
       </c>
-      <c r="E128" s="114"/>
-    </row>
-    <row r="129" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A129" s="81"/>
-      <c r="B129" s="84"/>
-      <c r="C129" s="67"/>
-      <c r="D129" s="26" t="s">
+      <c r="E129" s="66"/>
+    </row>
+    <row r="130" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A130" s="94"/>
+      <c r="B130" s="74"/>
+      <c r="C130" s="71"/>
+      <c r="D130" s="26" t="s">
         <v>200</v>
       </c>
-      <c r="E129" s="114"/>
-    </row>
-    <row r="130" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A130" s="81"/>
-      <c r="B130" s="84"/>
-      <c r="C130" s="67"/>
-      <c r="D130" s="28" t="s">
+      <c r="E130" s="66"/>
+    </row>
+    <row r="131" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A131" s="94"/>
+      <c r="B131" s="74"/>
+      <c r="C131" s="71"/>
+      <c r="D131" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="E130" s="114"/>
-    </row>
-    <row r="131" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A131" s="81"/>
-      <c r="B131" s="84"/>
-      <c r="C131" s="67" t="s">
+      <c r="E131" s="66"/>
+    </row>
+    <row r="132" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A132" s="94"/>
+      <c r="B132" s="74"/>
+      <c r="C132" s="71" t="s">
         <v>104</v>
       </c>
-      <c r="D131" s="26" t="s">
+      <c r="D132" s="26" t="s">
         <v>213</v>
       </c>
-      <c r="E131" s="114"/>
-    </row>
-    <row r="132" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A132" s="81"/>
-      <c r="B132" s="84"/>
-      <c r="C132" s="67"/>
-      <c r="D132" s="26" t="s">
+      <c r="E132" s="66"/>
+    </row>
+    <row r="133" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A133" s="94"/>
+      <c r="B133" s="74"/>
+      <c r="C133" s="71"/>
+      <c r="D133" s="26" t="s">
         <v>183</v>
       </c>
-      <c r="E132" s="114"/>
-    </row>
-    <row r="133" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A133" s="81"/>
-      <c r="B133" s="84"/>
-      <c r="C133" s="67"/>
-      <c r="D133" s="26" t="s">
+      <c r="E133" s="66"/>
+    </row>
+    <row r="134" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A134" s="94"/>
+      <c r="B134" s="74"/>
+      <c r="C134" s="71"/>
+      <c r="D134" s="26" t="s">
         <v>200</v>
       </c>
-      <c r="E133" s="114"/>
-    </row>
-    <row r="134" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A134" s="81"/>
-      <c r="B134" s="84"/>
-      <c r="C134" s="67"/>
-      <c r="D134" s="28" t="s">
+      <c r="E134" s="66"/>
+    </row>
+    <row r="135" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A135" s="94"/>
+      <c r="B135" s="74"/>
+      <c r="C135" s="71"/>
+      <c r="D135" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="E134" s="114"/>
-    </row>
-    <row r="135" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A135" s="81"/>
-      <c r="B135" s="84"/>
-      <c r="C135" s="86" t="s">
+      <c r="E135" s="66"/>
+    </row>
+    <row r="136" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A136" s="94"/>
+      <c r="B136" s="74"/>
+      <c r="C136" s="92" t="s">
         <v>195</v>
       </c>
-      <c r="D135" s="52" t="s">
+      <c r="D136" s="52" t="s">
         <v>183</v>
       </c>
-      <c r="E135" s="113"/>
-    </row>
-    <row r="136" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A136" s="81"/>
-      <c r="B136" s="84"/>
-      <c r="C136" s="87"/>
-      <c r="D136" s="52" t="s">
+      <c r="E136" s="65"/>
+    </row>
+    <row r="137" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A137" s="94"/>
+      <c r="B137" s="74"/>
+      <c r="C137" s="103"/>
+      <c r="D137" s="52" t="s">
         <v>201</v>
       </c>
-      <c r="E136" s="113"/>
-    </row>
-    <row r="137" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A137" s="82"/>
-      <c r="B137" s="85"/>
-      <c r="C137" s="88"/>
-      <c r="D137" s="53" t="s">
+      <c r="E137" s="65"/>
+    </row>
+    <row r="138" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A138" s="97"/>
+      <c r="B138" s="75"/>
+      <c r="C138" s="104"/>
+      <c r="D138" s="53" t="s">
         <v>202</v>
       </c>
-      <c r="E137" s="113"/>
-    </row>
-    <row r="138" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A138" s="80" t="s">
+      <c r="E138" s="65"/>
+    </row>
+    <row r="139" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A139" s="93" t="s">
         <v>105</v>
       </c>
-      <c r="B138" s="83" t="s">
+      <c r="B139" s="73" t="s">
         <v>106</v>
       </c>
-      <c r="C138" s="106" t="s">
+      <c r="C139" s="84" t="s">
         <v>107</v>
       </c>
-      <c r="D138" s="34" t="s">
+      <c r="D139" s="34" t="s">
         <v>183</v>
       </c>
-      <c r="E138" s="113"/>
-    </row>
-    <row r="139" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A139" s="81"/>
-      <c r="B139" s="84"/>
-      <c r="C139" s="109"/>
-      <c r="D139" s="34" t="s">
+      <c r="E139" s="65"/>
+    </row>
+    <row r="140" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A140" s="94"/>
+      <c r="B140" s="74"/>
+      <c r="C140" s="105"/>
+      <c r="D140" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="E139" s="113"/>
-    </row>
-    <row r="140" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A140" s="81"/>
-      <c r="B140" s="84"/>
-      <c r="C140" s="106" t="s">
+      <c r="E140" s="65"/>
+    </row>
+    <row r="141" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A141" s="94"/>
+      <c r="B141" s="74"/>
+      <c r="C141" s="84" t="s">
         <v>108</v>
       </c>
-      <c r="D140" s="34" t="s">
+      <c r="D141" s="34" t="s">
         <v>183</v>
       </c>
-      <c r="E140" s="113"/>
-    </row>
-    <row r="141" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A141" s="81"/>
-      <c r="B141" s="84"/>
-      <c r="C141" s="109"/>
-      <c r="D141" s="34" t="s">
+      <c r="E141" s="65"/>
+    </row>
+    <row r="142" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A142" s="94"/>
+      <c r="B142" s="74"/>
+      <c r="C142" s="105"/>
+      <c r="D142" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="E141" s="113"/>
-    </row>
-    <row r="142" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A142" s="81"/>
-      <c r="B142" s="84"/>
-      <c r="C142" s="5" t="s">
+      <c r="E142" s="65"/>
+    </row>
+    <row r="143" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A143" s="94"/>
+      <c r="B143" s="74"/>
+      <c r="C143" s="5" t="s">
         <v>109</v>
-      </c>
-      <c r="D142" s="34" t="s">
-        <v>209</v>
-      </c>
-      <c r="E142" s="113"/>
-    </row>
-    <row r="143" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A143" s="81"/>
-      <c r="B143" s="84"/>
-      <c r="C143" s="54" t="s">
-        <v>203</v>
       </c>
       <c r="D143" s="34" t="s">
         <v>209</v>
       </c>
-      <c r="E143" s="113"/>
+      <c r="E143" s="65"/>
     </row>
     <row r="144" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A144" s="81"/>
-      <c r="B144" s="84"/>
+      <c r="A144" s="94"/>
+      <c r="B144" s="74"/>
       <c r="C144" s="54" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D144" s="34" t="s">
         <v>209</v>
       </c>
-      <c r="E144" s="113"/>
+      <c r="E144" s="65"/>
     </row>
     <row r="145" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A145" s="81"/>
-      <c r="B145" s="84"/>
+      <c r="A145" s="94"/>
+      <c r="B145" s="74"/>
       <c r="C145" s="54" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D145" s="34" t="s">
         <v>209</v>
       </c>
-      <c r="E145" s="113"/>
+      <c r="E145" s="65"/>
     </row>
     <row r="146" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A146" s="81"/>
-      <c r="B146" s="84"/>
+      <c r="A146" s="94"/>
+      <c r="B146" s="74"/>
       <c r="C146" s="54" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D146" s="34" t="s">
         <v>209</v>
       </c>
-      <c r="E146" s="113"/>
+      <c r="E146" s="65"/>
     </row>
     <row r="147" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A147" s="81"/>
-      <c r="B147" s="84"/>
+      <c r="A147" s="94"/>
+      <c r="B147" s="74"/>
       <c r="C147" s="54" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D147" s="34" t="s">
         <v>209</v>
       </c>
-      <c r="E147" s="113"/>
+      <c r="E147" s="65"/>
     </row>
     <row r="148" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A148" s="81"/>
-      <c r="B148" s="84"/>
+      <c r="A148" s="94"/>
+      <c r="B148" s="74"/>
       <c r="C148" s="54" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D148" s="34" t="s">
         <v>209</v>
       </c>
-      <c r="E148" s="113"/>
-    </row>
-    <row r="149" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A149" s="82"/>
-      <c r="B149" s="85"/>
-      <c r="C149" s="55" t="s">
-        <v>110</v>
+      <c r="E148" s="65"/>
+    </row>
+    <row r="149" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A149" s="94"/>
+      <c r="B149" s="74"/>
+      <c r="C149" s="54" t="s">
+        <v>208</v>
       </c>
       <c r="D149" s="34" t="s">
         <v>209</v>
       </c>
-      <c r="E149" s="113"/>
-    </row>
-    <row r="150" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A150" s="75" t="s">
+      <c r="E149" s="65"/>
+    </row>
+    <row r="150" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A150" s="97"/>
+      <c r="B150" s="75"/>
+      <c r="C150" s="55" t="s">
+        <v>110</v>
+      </c>
+      <c r="D150" s="34" t="s">
+        <v>209</v>
+      </c>
+      <c r="E150" s="65"/>
+    </row>
+    <row r="151" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A151" s="99" t="s">
         <v>114</v>
       </c>
-      <c r="B150" s="77" t="s">
+      <c r="B151" s="101" t="s">
         <v>115</v>
       </c>
-      <c r="C150" s="79" t="s">
+      <c r="C151" s="98" t="s">
         <v>112</v>
       </c>
-      <c r="D150" s="34" t="s">
+      <c r="D151" s="34" t="s">
         <v>183</v>
       </c>
-      <c r="E150" s="113"/>
-    </row>
-    <row r="151" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A151" s="75"/>
-      <c r="B151" s="77"/>
-      <c r="C151" s="67"/>
-      <c r="D151" s="48" t="s">
+      <c r="E151" s="65"/>
+    </row>
+    <row r="152" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A152" s="99"/>
+      <c r="B152" s="101"/>
+      <c r="C152" s="71"/>
+      <c r="D152" s="48" t="s">
         <v>149</v>
       </c>
-      <c r="E151" s="113"/>
-    </row>
-    <row r="152" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A152" s="75"/>
-      <c r="B152" s="77"/>
-      <c r="C152" s="67" t="s">
+      <c r="E152" s="65"/>
+    </row>
+    <row r="153" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A153" s="99"/>
+      <c r="B153" s="101"/>
+      <c r="C153" s="71" t="s">
         <v>113</v>
       </c>
-      <c r="D152" s="32" t="s">
+      <c r="D153" s="32" t="s">
         <v>183</v>
       </c>
-      <c r="E152" s="113"/>
-    </row>
-    <row r="153" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A153" s="76"/>
-      <c r="B153" s="78"/>
-      <c r="C153" s="68"/>
-      <c r="D153" s="33" t="s">
+      <c r="E153" s="65"/>
+    </row>
+    <row r="154" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A154" s="100"/>
+      <c r="B154" s="102"/>
+      <c r="C154" s="96"/>
+      <c r="D154" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="E153" s="113"/>
-    </row>
-    <row r="154" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A154" s="63">
+      <c r="E154" s="65"/>
+    </row>
+    <row r="155" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A155" s="106">
         <v>21</v>
       </c>
-      <c r="B154" s="65" t="s">
+      <c r="B155" s="108" t="s">
         <v>116</v>
       </c>
-      <c r="C154" s="61" t="s">
+      <c r="C155" s="70" t="s">
         <v>117</v>
       </c>
-      <c r="D154" s="31" t="s">
+      <c r="D155" s="31" t="s">
         <v>196</v>
       </c>
-      <c r="E154" s="113"/>
-    </row>
-    <row r="155" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A155" s="64"/>
-      <c r="B155" s="66"/>
-      <c r="C155" s="62"/>
-      <c r="D155" s="35" t="s">
+      <c r="E155" s="65"/>
+    </row>
+    <row r="156" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A156" s="107"/>
+      <c r="B156" s="109"/>
+      <c r="C156" s="72"/>
+      <c r="D156" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="E155" s="113"/>
-    </row>
-    <row r="156" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A156" s="69">
+      <c r="E156" s="65"/>
+    </row>
+    <row r="157" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A157" s="110">
         <v>22</v>
       </c>
-      <c r="B156" s="72" t="s">
+      <c r="B157" s="113" t="s">
         <v>118</v>
       </c>
-      <c r="C156" s="61" t="s">
+      <c r="C157" s="70" t="s">
         <v>119</v>
       </c>
-      <c r="D156" s="31" t="s">
+      <c r="D157" s="31" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="157" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A157" s="70"/>
-      <c r="B157" s="73"/>
-      <c r="C157" s="67"/>
-      <c r="D157" s="32" t="s">
+      <c r="E157" s="65"/>
+    </row>
+    <row r="158" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A158" s="111"/>
+      <c r="B158" s="114"/>
+      <c r="C158" s="71"/>
+      <c r="D158" s="32" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="158" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A158" s="70"/>
-      <c r="B158" s="73"/>
-      <c r="C158" s="5" t="s">
+      <c r="E158" s="65"/>
+    </row>
+    <row r="159" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A159" s="111"/>
+      <c r="B159" s="114"/>
+      <c r="C159" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="D158" s="32" t="s">
+      <c r="D159" s="32" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="159" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A159" s="70"/>
-      <c r="B159" s="73"/>
-      <c r="C159" s="67" t="s">
+      <c r="E159" s="65"/>
+    </row>
+    <row r="160" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A160" s="111"/>
+      <c r="B160" s="114"/>
+      <c r="C160" s="71" t="s">
         <v>121</v>
       </c>
-      <c r="D159" s="32" t="s">
+      <c r="D160" s="32" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="160" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A160" s="71"/>
-      <c r="B160" s="74"/>
-      <c r="C160" s="68"/>
-      <c r="D160" s="33" t="s">
+      <c r="E160" s="65"/>
+    </row>
+    <row r="161" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A161" s="112"/>
+      <c r="B161" s="115"/>
+      <c r="C161" s="96"/>
+      <c r="D161" s="33" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="161" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A161" s="19" t="s">
+      <c r="E161" s="65"/>
+    </row>
+    <row r="162" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A162" s="19" t="s">
         <v>122</v>
       </c>
-      <c r="B161" s="4" t="s">
+      <c r="B162" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="C161" s="4" t="s">
+      <c r="C162" s="4" t="s">
         <v>67</v>
-      </c>
-      <c r="D161" s="36" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="162" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A162" s="19" t="s">
-        <v>124</v>
-      </c>
-      <c r="B162" s="4"/>
-      <c r="C162" s="4" t="s">
-        <v>125</v>
       </c>
       <c r="D162" s="36" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="163" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E162" s="65"/>
+    </row>
+    <row r="163" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A163" s="19" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B163" s="4"/>
       <c r="C163" s="4" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D163" s="36" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="164" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>67</v>
+      </c>
+      <c r="E163" s="65"/>
+    </row>
+    <row r="164" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A164" s="19" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B164" s="4"/>
       <c r="C164" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D164" s="36" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="165" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+      <c r="E164" s="65"/>
+    </row>
+    <row r="165" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A165" s="19" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B165" s="4"/>
       <c r="C165" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="D165" s="36" t="s">
+        <v>67</v>
+      </c>
+      <c r="E165" s="65"/>
+    </row>
+    <row r="166" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A166" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="B166" s="4"/>
+      <c r="C166" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="D165" s="36"/>
-    </row>
-    <row r="166" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A166" s="22"/>
-      <c r="B166" s="22"/>
-      <c r="C166" s="22"/>
-      <c r="D166" s="24"/>
-    </row>
-    <row r="167" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D166" s="36"/>
+      <c r="E166" s="65"/>
+    </row>
+    <row r="167" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A167" s="22"/>
       <c r="B167" s="22"/>
       <c r="C167" s="22"/>
       <c r="D167" s="24"/>
     </row>
-    <row r="168" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A168" s="22"/>
       <c r="B168" s="22"/>
       <c r="C168" s="22"/>
       <c r="D168" s="24"/>
     </row>
-    <row r="169" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A169" s="22"/>
       <c r="B169" s="22"/>
       <c r="C169" s="22"/>
       <c r="D169" s="24"/>
     </row>
-    <row r="170" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A170" s="22"/>
       <c r="B170" s="22"/>
       <c r="C170" s="22"/>
       <c r="D170" s="24"/>
     </row>
-    <row r="171" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A171" s="22"/>
       <c r="B171" s="22"/>
       <c r="C171" s="22"/>
       <c r="D171" s="24"/>
     </row>
-    <row r="172" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A172" s="22"/>
       <c r="B172" s="22"/>
       <c r="C172" s="22"/>
       <c r="D172" s="24"/>
     </row>
-    <row r="173" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A173" s="22"/>
       <c r="B173" s="22"/>
       <c r="C173" s="22"/>
       <c r="D173" s="24"/>
     </row>
-    <row r="174" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A174" s="22"/>
       <c r="B174" s="22"/>
       <c r="C174" s="22"/>
       <c r="D174" s="24"/>
     </row>
-    <row r="175" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A175" s="22"/>
       <c r="B175" s="22"/>
       <c r="C175" s="22"/>
       <c r="D175" s="24"/>
     </row>
-    <row r="176" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A176" s="22"/>
       <c r="B176" s="22"/>
       <c r="C176" s="22"/>
@@ -5219,6 +5259,7 @@
       <c r="A277" s="22"/>
       <c r="B277" s="22"/>
       <c r="C277" s="22"/>
+      <c r="D277" s="24"/>
     </row>
     <row r="278" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A278" s="22"/>
@@ -5295,20 +5336,67 @@
       <c r="B292" s="22"/>
       <c r="C292" s="22"/>
     </row>
+    <row r="293" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A293" s="22"/>
+      <c r="B293" s="22"/>
+      <c r="C293" s="22"/>
+    </row>
   </sheetData>
   <mergeCells count="83">
-    <mergeCell ref="A25:A27"/>
-    <mergeCell ref="B25:B27"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="B138:B149"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="C51:C52"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="C55:C56"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="C60:C61"/>
-    <mergeCell ref="C62:C63"/>
-    <mergeCell ref="C64:C65"/>
+    <mergeCell ref="C155:C156"/>
+    <mergeCell ref="A155:A156"/>
+    <mergeCell ref="B155:B156"/>
+    <mergeCell ref="C157:C158"/>
+    <mergeCell ref="C160:C161"/>
+    <mergeCell ref="A157:A161"/>
+    <mergeCell ref="B157:B161"/>
+    <mergeCell ref="C128:C131"/>
+    <mergeCell ref="C132:C135"/>
+    <mergeCell ref="C153:C154"/>
+    <mergeCell ref="A151:A154"/>
+    <mergeCell ref="B151:B154"/>
+    <mergeCell ref="C151:C152"/>
+    <mergeCell ref="A119:A138"/>
+    <mergeCell ref="B119:B138"/>
+    <mergeCell ref="C136:C138"/>
+    <mergeCell ref="C119:C121"/>
+    <mergeCell ref="C124:C125"/>
+    <mergeCell ref="C126:C127"/>
+    <mergeCell ref="C122:C123"/>
+    <mergeCell ref="C139:C140"/>
+    <mergeCell ref="C141:C142"/>
+    <mergeCell ref="A139:A150"/>
+    <mergeCell ref="C101:C102"/>
+    <mergeCell ref="C103:C104"/>
+    <mergeCell ref="C105:C106"/>
+    <mergeCell ref="A99:A118"/>
+    <mergeCell ref="B99:B118"/>
+    <mergeCell ref="C107:C108"/>
+    <mergeCell ref="C109:C110"/>
+    <mergeCell ref="C111:C112"/>
+    <mergeCell ref="C113:C114"/>
+    <mergeCell ref="C115:C116"/>
+    <mergeCell ref="C117:C118"/>
+    <mergeCell ref="C95:C96"/>
+    <mergeCell ref="C97:C98"/>
+    <mergeCell ref="A92:A98"/>
+    <mergeCell ref="B92:B98"/>
+    <mergeCell ref="C99:C100"/>
+    <mergeCell ref="A59:A73"/>
+    <mergeCell ref="B59:B73"/>
+    <mergeCell ref="A90:A91"/>
+    <mergeCell ref="B90:B91"/>
+    <mergeCell ref="C93:C94"/>
+    <mergeCell ref="A77:A78"/>
+    <mergeCell ref="B77:B78"/>
+    <mergeCell ref="C88:C89"/>
+    <mergeCell ref="A81:A89"/>
+    <mergeCell ref="B81:B89"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="C38:C40"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="C47:C48"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="B14:B21"/>
@@ -5322,64 +5410,22 @@
     <mergeCell ref="C12:C13"/>
     <mergeCell ref="B10:B13"/>
     <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A25:A27"/>
+    <mergeCell ref="B25:B27"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="B139:B150"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="C51:C52"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="C55:C56"/>
+    <mergeCell ref="C57:C58"/>
+    <mergeCell ref="C60:C61"/>
+    <mergeCell ref="C62:C63"/>
+    <mergeCell ref="C64:C65"/>
     <mergeCell ref="C31:C32"/>
     <mergeCell ref="C33:C34"/>
     <mergeCell ref="A28:A58"/>
     <mergeCell ref="B28:B58"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="C38:C40"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="C45:C46"/>
-    <mergeCell ref="C47:C48"/>
-    <mergeCell ref="A59:A73"/>
-    <mergeCell ref="B59:B73"/>
-    <mergeCell ref="A89:A90"/>
-    <mergeCell ref="B89:B90"/>
-    <mergeCell ref="C92:C93"/>
-    <mergeCell ref="A76:A77"/>
-    <mergeCell ref="B76:B77"/>
-    <mergeCell ref="C87:C88"/>
-    <mergeCell ref="A80:A88"/>
-    <mergeCell ref="B80:B88"/>
-    <mergeCell ref="C94:C95"/>
-    <mergeCell ref="C96:C97"/>
-    <mergeCell ref="A91:A97"/>
-    <mergeCell ref="B91:B97"/>
-    <mergeCell ref="C98:C99"/>
-    <mergeCell ref="C100:C101"/>
-    <mergeCell ref="C102:C103"/>
-    <mergeCell ref="C104:C105"/>
-    <mergeCell ref="A98:A117"/>
-    <mergeCell ref="B98:B117"/>
-    <mergeCell ref="C106:C107"/>
-    <mergeCell ref="C108:C109"/>
-    <mergeCell ref="C110:C111"/>
-    <mergeCell ref="C112:C113"/>
-    <mergeCell ref="C114:C115"/>
-    <mergeCell ref="C116:C117"/>
-    <mergeCell ref="C127:C130"/>
-    <mergeCell ref="C131:C134"/>
-    <mergeCell ref="C152:C153"/>
-    <mergeCell ref="A150:A153"/>
-    <mergeCell ref="B150:B153"/>
-    <mergeCell ref="C150:C151"/>
-    <mergeCell ref="A118:A137"/>
-    <mergeCell ref="B118:B137"/>
-    <mergeCell ref="C135:C137"/>
-    <mergeCell ref="C118:C120"/>
-    <mergeCell ref="C123:C124"/>
-    <mergeCell ref="C125:C126"/>
-    <mergeCell ref="C121:C122"/>
-    <mergeCell ref="C138:C139"/>
-    <mergeCell ref="C140:C141"/>
-    <mergeCell ref="A138:A149"/>
-    <mergeCell ref="C154:C155"/>
-    <mergeCell ref="A154:A155"/>
-    <mergeCell ref="B154:B155"/>
-    <mergeCell ref="C156:C157"/>
-    <mergeCell ref="C159:C160"/>
-    <mergeCell ref="A156:A160"/>
-    <mergeCell ref="B156:B160"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>

</xml_diff>